<commit_message>
doc improvements in sequence documentation
add lstm related QAs and fix in sequence pptx
</commit_message>
<xml_diff>
--- a/my_notes/sequence_models/explainers_w1_rnn_calculations.xlsx
+++ b/my_notes/sequence_models/explainers_w1_rnn_calculations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/takis/Documents/sckool/notes-deep-learning/MyMaterial/sequence_models/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/takis/Documents/sckool/notes-deep-learning/my_notes/sequence_models/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB43016F-BD96-BE47-A038-E167F01FA24B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{657A5B52-A500-114E-92A6-E34684B58BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16060" activeTab="2" xr2:uid="{EA0C6A45-9098-3045-B6B2-2B0794646868}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="101">
   <si>
     <t>Input Dim</t>
   </si>
@@ -448,9 +448,6 @@
     <t>(N, L, Hin)</t>
   </si>
   <si>
-    <t>N</t>
-  </si>
-  <si>
     <t>X{1}_t=1</t>
   </si>
   <si>
@@ -479,6 +476,1268 @@
   </si>
   <si>
     <t>Check : explainers_w1_rnn_calculations.py</t>
+  </si>
+  <si>
+    <t>(N, L, Hin) = (2,4,4)</t>
+  </si>
+  <si>
+    <t>https://docs.pytorch.org/docs/stable/generated/torch.nn.LSTM.html</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>.],</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>.],</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>.]],</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>.],</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>.],</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>.],</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>.]]])</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">., </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>.],</t>
+    </r>
+  </si>
+  <si>
+    <t>tensor([[</t>
+  </si>
+  <si>
+    <t>[2, 4, 4]</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.7475</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.3686</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.4642</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>],</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.2070</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.6717</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.3048</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>],</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.9873</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.7887</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.6557</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>],</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.9889</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.6644</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.3555</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>],</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.9377</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.5384</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.1204</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>],</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">[ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.5970</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.0218</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>0.7883</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>],</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>grad_fn</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>=&lt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>TransposeBackward1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>[2, 4, 3]</t>
+  </si>
+  <si>
+    <t>output</t>
+  </si>
+  <si>
+    <t>hn</t>
+  </si>
+  <si>
+    <t>[1, 2, 3]</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFD19A66"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>grad_fn</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>=&lt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>StackBackward0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFC678DD"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFABB2BF"/>
+        <rFont val="Menlo"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>(N)</t>
+  </si>
+  <si>
+    <t>Sequence Length (L)</t>
+  </si>
+  <si>
+    <t>(N, L, Hout)</t>
+  </si>
+  <si>
+    <t>input</t>
+  </si>
+  <si>
+    <t>https://docs.pytorch.org/docs/stable/generated/torch.nn.RNN.html</t>
+  </si>
+  <si>
+    <t>(N, L, Hout) = (2,4,3)</t>
+  </si>
+  <si>
+    <t>hx, h_n</t>
+  </si>
+  <si>
+    <t>(num layers, N, Hout) = (1,2,3)</t>
+  </si>
+  <si>
+    <t>[-0.9492, -0.9351, -0.6876]],</t>
+  </si>
+  <si>
+    <t>[-0.2894, -0.4460, -0.6800]]]</t>
+  </si>
+  <si>
+    <t>[-0.9492, -0.9351, -0.6876],</t>
+  </si>
+  <si>
+    <t>Hidden State (Hout)</t>
+  </si>
+  <si>
+    <t>Input (Hin)</t>
   </si>
 </sst>
 </file>
@@ -489,7 +1748,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
     <numFmt numFmtId="165" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -543,8 +1802,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFC00000"/>
+      <name val="Menlo"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -599,6 +1881,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -624,10 +1912,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -690,11 +1979,21 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1579,14 +2878,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>180212</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>19539</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>10226</xdr:rowOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>10227</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1623,14 +2922,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>58616</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>19538</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>155331</xdr:rowOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>155330</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1667,13 +2966,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>58616</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>63500</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>156308</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -1721,13 +3020,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>58616</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>63500</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>156308</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -1775,13 +3074,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>58616</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>156308</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>63500</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>117232</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -1829,13 +3128,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>39076</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:row>30</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>39076</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -1886,13 +3185,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>39076</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>34</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>39076</xdr:colOff>
-      <xdr:row>35</xdr:row>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>-1</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -1943,13 +3242,13 @@
     <xdr:from>
       <xdr:col>13</xdr:col>
       <xdr:colOff>4884</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>145520</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
       <xdr:colOff>727604</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>145520</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -2000,13 +3299,13 @@
     <xdr:from>
       <xdr:col>12</xdr:col>
       <xdr:colOff>395409</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>139170</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>806979</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>139170</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -2057,13 +3356,13 @@
     <xdr:from>
       <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>132290</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>41153</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>132290</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -2114,13 +3413,13 @@
     <xdr:from>
       <xdr:col>19</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>132290</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>41153</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>132290</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -2171,13 +3470,13 @@
     <xdr:from>
       <xdr:col>22</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>132290</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>41154</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>132290</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -2202,6 +3501,63 @@
         <a:ln w="28575">
           <a:solidFill>
             <a:srgbClr val="C00000"/>
+          </a:solidFill>
+          <a:headEnd type="triangle"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>223297</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>139561</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>223297</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>195385</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="3" name="Straight Arrow Connector 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{580A86D5-BF6D-1B42-A36B-D10AC5F96FBA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="8317802" y="1186264"/>
+          <a:ext cx="0" cy="893187"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="28575">
+          <a:solidFill>
+            <a:srgbClr val="00B0F0"/>
           </a:solidFill>
           <a:headEnd type="triangle"/>
           <a:tailEnd type="triangle"/>
@@ -3333,15 +4689,15 @@
         <v>0.99927735073811652</v>
       </c>
       <c r="X18" s="12">
-        <f>V36</f>
+        <f t="shared" ref="X18:X23" si="1">V36</f>
         <v>0.99815815900919547</v>
       </c>
       <c r="Z18" s="12">
-        <f>X36</f>
+        <f t="shared" ref="Z18:Z23" si="2">X36</f>
         <v>0.99999994653002799</v>
       </c>
       <c r="AB18" s="12">
-        <f>Z36</f>
+        <f t="shared" ref="AB18:AB23" si="3">Z36</f>
         <v>0.99936272232463363</v>
       </c>
     </row>
@@ -3374,7 +4730,7 @@
         <v>0</v>
       </c>
       <c r="T19" s="12">
-        <f t="shared" ref="T19:T23" si="1">R37</f>
+        <f t="shared" ref="T19:T23" si="4">R37</f>
         <v>-0.76159415595576485</v>
       </c>
       <c r="V19" s="12">
@@ -3382,15 +4738,15 @@
         <v>0.99990243158805026</v>
       </c>
       <c r="X19" s="12">
-        <f>V37</f>
+        <f t="shared" si="1"/>
         <v>4.9755932948084801E-3</v>
       </c>
       <c r="Z19" s="12">
-        <f>X37</f>
+        <f t="shared" si="2"/>
         <v>-0.94681701559291809</v>
       </c>
       <c r="AB19" s="12">
-        <f>Z37</f>
+        <f t="shared" si="3"/>
         <v>0.99989932710479446</v>
       </c>
     </row>
@@ -3423,7 +4779,7 @@
         <v>0</v>
       </c>
       <c r="T20" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0.76159415595576485</v>
       </c>
       <c r="V20" s="12">
@@ -3431,15 +4787,15 @@
         <v>0.99883923596754132</v>
       </c>
       <c r="X20" s="12">
-        <f>V38</f>
+        <f t="shared" si="1"/>
         <v>0.99507991252818306</v>
       </c>
       <c r="Z20" s="12">
-        <f>X38</f>
+        <f t="shared" si="2"/>
         <v>0.97550374173012133</v>
       </c>
       <c r="AB20" s="12">
-        <f>Z38</f>
+        <f t="shared" si="3"/>
         <v>0.99926256554001103</v>
       </c>
     </row>
@@ -3472,7 +4828,7 @@
         <v>0</v>
       </c>
       <c r="T21" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0.99932929973906692</v>
       </c>
       <c r="V21" s="12">
@@ -3480,15 +4836,15 @@
         <v>-0.50834989944641529</v>
       </c>
       <c r="X21" s="12">
-        <f>V39</f>
+        <f t="shared" si="1"/>
         <v>0.75654273933495453</v>
       </c>
       <c r="Z21" s="12">
-        <f>X39</f>
+        <f t="shared" si="2"/>
         <v>0.99997861293651025</v>
       </c>
       <c r="AB21" s="12">
-        <f>Z39</f>
+        <f t="shared" si="3"/>
         <v>-0.73765305319017993</v>
       </c>
     </row>
@@ -3521,7 +4877,7 @@
         <v>0</v>
       </c>
       <c r="T22" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>-0.76159415595576485</v>
       </c>
       <c r="V22" s="12">
@@ -3529,15 +4885,15 @@
         <v>0.99993943236914828</v>
       </c>
       <c r="X22" s="12">
-        <f>V40</f>
+        <f t="shared" si="1"/>
         <v>-0.7590206427231786</v>
       </c>
       <c r="Z22" s="12">
-        <f>X40</f>
+        <f t="shared" si="2"/>
         <v>-0.99535311804591431</v>
       </c>
       <c r="AB22" s="12">
-        <f>Z40</f>
+        <f t="shared" si="3"/>
         <v>0.99991300777743042</v>
       </c>
     </row>
@@ -3570,7 +4926,7 @@
         <v>0</v>
       </c>
       <c r="T23" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0.96402758007581701</v>
       </c>
       <c r="V23" s="12">
@@ -3578,15 +4934,15 @@
         <v>-0.99506136642620702</v>
       </c>
       <c r="X23" s="12">
-        <f>V41</f>
+        <f t="shared" si="1"/>
         <v>0.96388997852092517</v>
       </c>
       <c r="Z23" s="12">
-        <f>X41</f>
+        <f t="shared" si="2"/>
         <v>0.99690150300965796</v>
       </c>
       <c r="AB23" s="12">
-        <f>Z41</f>
+        <f t="shared" si="3"/>
         <v>-0.99524677109355042</v>
       </c>
     </row>
@@ -3849,27 +5205,27 @@
         <v>1</v>
       </c>
       <c r="R36" s="13">
-        <f t="shared" ref="R36:X38" si="2">TANH(R27)</f>
+        <f t="shared" ref="R36:X38" si="5">TANH(R27)</f>
         <v>0.99932929973906692</v>
       </c>
       <c r="T36" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.99927735073811652</v>
       </c>
       <c r="V36" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.99815815900919547</v>
       </c>
       <c r="X36" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.99999994653002799</v>
       </c>
       <c r="Z36" s="13">
-        <f t="shared" ref="Z36:AB36" si="3">TANH(Z27)</f>
+        <f t="shared" ref="Z36:AB36" si="6">TANH(Z27)</f>
         <v>0.99936272232463363</v>
       </c>
       <c r="AB36" s="13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>0.99960566099102655</v>
       </c>
     </row>
@@ -3878,27 +5234,27 @@
         <v>0</v>
       </c>
       <c r="R37" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>-0.76159415595576485</v>
       </c>
       <c r="T37" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.99990243158805026</v>
       </c>
       <c r="V37" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>4.9755932948084801E-3</v>
       </c>
       <c r="X37" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>-0.94681701559291809</v>
       </c>
       <c r="Z37" s="13">
-        <f t="shared" ref="Z37:AB37" si="4">TANH(Z28)</f>
+        <f t="shared" ref="Z37:AB37" si="7">TANH(Z28)</f>
         <v>0.99989932710479446</v>
       </c>
       <c r="AB37" s="13">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.99510156181258513</v>
       </c>
     </row>
@@ -3907,27 +5263,27 @@
         <v>1</v>
       </c>
       <c r="R38" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.76159415595576485</v>
       </c>
       <c r="T38" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.99883923596754132</v>
       </c>
       <c r="V38" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.99507991252818306</v>
       </c>
       <c r="X38" s="13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.97550374173012133</v>
       </c>
       <c r="Z38" s="13">
-        <f t="shared" ref="Z38:AB38" si="5">TANH(Z29)</f>
+        <f t="shared" ref="Z38:AB38" si="8">TANH(Z29)</f>
         <v>0.99926256554001103</v>
       </c>
       <c r="AB38" s="13">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>0.99508614006301643</v>
       </c>
     </row>
@@ -3936,27 +5292,27 @@
         <v>1</v>
       </c>
       <c r="R39" s="13">
-        <f t="shared" ref="R39:X39" si="6">TANH(R30)</f>
+        <f t="shared" ref="R39:X39" si="9">TANH(R30)</f>
         <v>0.99932929973906692</v>
       </c>
       <c r="T39" s="13">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>-0.50834989944641529</v>
       </c>
       <c r="V39" s="13">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.75654273933495453</v>
       </c>
       <c r="X39" s="13">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.99997861293651025</v>
       </c>
       <c r="Z39" s="13">
-        <f t="shared" ref="Z39:AB39" si="7">TANH(Z30)</f>
+        <f t="shared" ref="Z39:AB39" si="10">TANH(Z30)</f>
         <v>-0.73765305319017993</v>
       </c>
       <c r="AB39" s="13">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>-0.98581333041235719</v>
       </c>
     </row>
@@ -3965,27 +5321,27 @@
         <v>0</v>
       </c>
       <c r="R40" s="13">
-        <f t="shared" ref="R40:X40" si="8">TANH(R31)</f>
+        <f t="shared" ref="R40:X40" si="11">TANH(R31)</f>
         <v>-0.76159415595576485</v>
       </c>
       <c r="T40" s="13">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.99993943236914828</v>
       </c>
       <c r="V40" s="13">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>-0.7590206427231786</v>
       </c>
       <c r="X40" s="13">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>-0.99535311804591431</v>
       </c>
       <c r="Z40" s="13">
-        <f t="shared" ref="Z40:AB40" si="9">TANH(Z31)</f>
+        <f t="shared" ref="Z40:AB40" si="12">TANH(Z31)</f>
         <v>0.99991300777743042</v>
       </c>
       <c r="AB40" s="13">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0.9644134536071256</v>
       </c>
     </row>
@@ -3994,27 +5350,27 @@
         <v>-1</v>
       </c>
       <c r="R41" s="13">
-        <f t="shared" ref="R41:X41" si="10">TANH(R32)</f>
+        <f t="shared" ref="R41:X41" si="13">TANH(R32)</f>
         <v>0.96402758007581701</v>
       </c>
       <c r="T41" s="13">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>-0.99506136642620702</v>
       </c>
       <c r="V41" s="13">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.96388997852092517</v>
       </c>
       <c r="X41" s="13">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.99690150300965796</v>
       </c>
       <c r="Z41" s="13">
-        <f t="shared" ref="Z41:AB41" si="11">TANH(Z32)</f>
+        <f t="shared" ref="Z41:AB41" si="14">TANH(Z32)</f>
         <v>-0.99524677109355042</v>
       </c>
       <c r="AB41" s="13">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>-0.76220735121980276</v>
       </c>
     </row>
@@ -4441,23 +5797,23 @@
         <v>0.61309952879809837</v>
       </c>
       <c r="T58" s="6">
-        <f t="shared" ref="T58:AB58" si="12">EXP(T45)</f>
+        <f t="shared" ref="T58:AB58" si="15">EXP(T45)</f>
         <v>147.34433806643816</v>
       </c>
       <c r="V58" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.61418641652494521</v>
       </c>
       <c r="X58" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.37246660376219043</v>
       </c>
       <c r="Z58" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>147.40161755688243</v>
       </c>
       <c r="AB58" s="6">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>108.83698816591154</v>
       </c>
     </row>
@@ -4467,27 +5823,27 @@
       </c>
       <c r="K59"/>
       <c r="R59" s="6">
-        <f t="shared" ref="R59:AB59" si="13">EXP(R46)</f>
+        <f t="shared" ref="R59:AB59" si="16">EXP(R46)</f>
         <v>0.46692148772244257</v>
       </c>
       <c r="T59" s="6">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>2.7180166229558611</v>
       </c>
       <c r="V59" s="6">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1.0049879921144249</v>
       </c>
       <c r="X59" s="6">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.38797397529401628</v>
       </c>
       <c r="Z59" s="6">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>2.7180081849318638</v>
       </c>
       <c r="AB59" s="6">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>2.7049990519359155</v>
       </c>
     </row>
@@ -4497,27 +5853,27 @@
       </c>
       <c r="K60"/>
       <c r="R60" s="6">
-        <f t="shared" ref="R60:AB60" si="14">EXP(R47)</f>
+        <f t="shared" ref="R60:AB60" si="17">EXP(R47)</f>
         <v>1.6098499692090575</v>
       </c>
       <c r="T60" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>54.552100389850118</v>
       </c>
       <c r="V60" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1.6162632896038467</v>
       </c>
       <c r="X60" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1.0093370310641705</v>
       </c>
       <c r="Z60" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>54.553874584098324</v>
       </c>
       <c r="AB60" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>50.827246956380478</v>
       </c>
     </row>
@@ -4527,27 +5883,27 @@
       </c>
       <c r="K61"/>
       <c r="R61" s="6">
-        <f t="shared" ref="R61:AB61" si="15">EXP(R48)</f>
+        <f t="shared" ref="R61:AB61" si="18">EXP(R48)</f>
         <v>7.384101918647767</v>
       </c>
       <c r="T61" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>1.635011929337661</v>
       </c>
       <c r="V61" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>5.7923769802525218</v>
       </c>
       <c r="X61" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>7.3888980704086222</v>
       </c>
       <c r="Z61" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>1.2999774872399623</v>
       </c>
       <c r="AB61" s="6">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>1.0142877779491526</v>
       </c>
     </row>
@@ -4557,27 +5913,27 @@
       </c>
       <c r="K62"/>
       <c r="R62" s="6">
-        <f t="shared" ref="R62:AB62" si="16">EXP(R49)</f>
+        <f t="shared" ref="R62:AB62" si="19">EXP(R49)</f>
         <v>1.2683732118033044</v>
       </c>
       <c r="T62" s="6">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>7.3832711311105825</v>
       </c>
       <c r="V62" s="6">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1.270153191324169</v>
       </c>
       <c r="X62" s="6">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1.0046576417342123</v>
       </c>
       <c r="Z62" s="6">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>7.3837063655833051</v>
       </c>
       <c r="AB62" s="6">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>7.127917489812055</v>
       </c>
     </row>
@@ -4587,27 +5943,27 @@
       </c>
       <c r="K63"/>
       <c r="R63" s="6">
-        <f t="shared" ref="R63:AB63" si="17">EXP(R50)</f>
+        <f t="shared" ref="R63:AB63" si="20">EXP(R50)</f>
         <v>3.3282060134402771</v>
       </c>
       <c r="T63" s="6">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>2.7314731120882088</v>
       </c>
       <c r="V63" s="6">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>7.1625464831633785</v>
       </c>
       <c r="X63" s="6">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>2.8578925638234933</v>
       </c>
       <c r="Z63" s="6">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>2.7309582529413188</v>
       </c>
       <c r="AB63" s="6">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>3.4311456377751082</v>
       </c>
     </row>
@@ -4617,27 +5973,27 @@
       </c>
       <c r="K64"/>
       <c r="R64" s="6">
-        <f t="shared" ref="R64:AB64" si="18">EXP(R51)</f>
+        <f t="shared" ref="R64:AB64" si="21">EXP(R51)</f>
         <v>0.5922307070424917</v>
       </c>
       <c r="T64" s="6">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>4.4437204489002173</v>
       </c>
       <c r="V64" s="6">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>1.0025008117325958</v>
       </c>
       <c r="X64" s="6">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>0.38977270373201051</v>
       </c>
       <c r="Z64" s="6">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>3.5330420899927395</v>
       </c>
       <c r="AB64" s="6">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>2.6477273943105399</v>
       </c>
     </row>
@@ -4647,27 +6003,27 @@
       </c>
       <c r="K65"/>
       <c r="R65" s="6">
-        <f t="shared" ref="R65:AB65" si="19">EXP(R52)</f>
+        <f t="shared" ref="R65:AB65" si="22">EXP(R52)</f>
         <v>50.774002404141633</v>
       </c>
       <c r="T65" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>1.649164894523069</v>
       </c>
       <c r="V65" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>108.24294615292001</v>
       </c>
       <c r="X65" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>55.838765203569679</v>
       </c>
       <c r="Z65" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>1.3112951294635624</v>
       </c>
       <c r="AB65" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>1.6160092256487064</v>
       </c>
     </row>
@@ -4677,27 +6033,27 @@
       </c>
       <c r="K66"/>
       <c r="R66" s="6">
-        <f t="shared" ref="R66:AB66" si="20">EXP(R53)</f>
+        <f t="shared" ref="R66:AB66" si="23">EXP(R53)</f>
         <v>0.27652524280719426</v>
       </c>
       <c r="T66" s="6">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>12.078552955505545</v>
       </c>
       <c r="V66" s="6">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0.46929535553225704</v>
       </c>
       <c r="X66" s="6">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0.14405722842357441</v>
       </c>
       <c r="Z66" s="6">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>9.602968692481415</v>
       </c>
       <c r="AB66" s="6">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>6.9456470430643327</v>
       </c>
     </row>
@@ -4707,27 +6063,27 @@
       </c>
       <c r="K67"/>
       <c r="R67" s="6">
-        <f t="shared" ref="R67:AB67" si="21">EXP(R54)</f>
+        <f t="shared" ref="R67:AB67" si="24">EXP(R54)</f>
         <v>5.8100086238425401</v>
       </c>
       <c r="T67" s="6">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>54.350290390182302</v>
       </c>
       <c r="V67" s="6">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>9.2591630329338752</v>
       </c>
       <c r="X67" s="6">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>7.0685417868297948</v>
       </c>
       <c r="Z67" s="6">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>54.40882178235379</v>
       </c>
       <c r="AB67" s="6">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>52.112389182851281</v>
       </c>
     </row>
@@ -4747,257 +6103,257 @@
         <v>8.5007115089178863E-3</v>
       </c>
       <c r="T71" s="5">
-        <f t="shared" ref="T71:AB71" si="22">T58/SUM(T$58:T$67)</f>
+        <f t="shared" ref="T71:AB71" si="25">T58/SUM(T$58:T$67)</f>
         <v>0.51004329977632679</v>
       </c>
       <c r="V71" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>4.5016969900116468E-3</v>
       </c>
       <c r="X71" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>4.871241092749677E-3</v>
       </c>
       <c r="Z71" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>0.51729981266764491</v>
       </c>
       <c r="AB71" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>0.45871613046921306</v>
       </c>
     </row>
     <row r="72" spans="9:28" x14ac:dyDescent="0.2">
       <c r="R72" s="5">
-        <f t="shared" ref="R72:AB80" si="23">R59/SUM(R$58:R$67)</f>
+        <f t="shared" ref="R72:AB80" si="26">R59/SUM(R$58:R$67)</f>
         <v>6.473932335626255E-3</v>
       </c>
       <c r="T72" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>9.4086151216358545E-3</v>
       </c>
       <c r="V72" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>7.3660883688976969E-3</v>
       </c>
       <c r="X72" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>5.0740516123596365E-3</v>
       </c>
       <c r="Z72" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>9.538736061371865E-3</v>
       </c>
       <c r="AB72" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1.1400781287106291E-2</v>
       </c>
     </row>
     <row r="73" spans="9:28" x14ac:dyDescent="0.2">
       <c r="R73" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>2.2320797061635235E-2</v>
       </c>
       <c r="T73" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0.188836121276833</v>
       </c>
       <c r="V73" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1.1846448228280617E-2</v>
       </c>
       <c r="X73" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1.3200442596708446E-2</v>
       </c>
       <c r="Z73" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0.19145454147921992</v>
       </c>
       <c r="AB73" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0.21422200705050784</v>
       </c>
     </row>
     <row r="74" spans="9:28" x14ac:dyDescent="0.2">
       <c r="R74" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0.10238161540577979</v>
       </c>
       <c r="T74" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>5.6597144522582063E-3</v>
       </c>
       <c r="V74" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>4.245539353434475E-2</v>
       </c>
       <c r="X74" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>9.6634446007121427E-2</v>
       </c>
       <c r="Z74" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>4.562216628062974E-3</v>
       </c>
       <c r="AB74" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>4.2749268656147674E-3</v>
       </c>
     </row>
     <row r="75" spans="9:28" x14ac:dyDescent="0.2">
       <c r="R75" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1.7586173619014753E-2</v>
       </c>
       <c r="T75" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>2.5557737883059508E-2</v>
       </c>
       <c r="V75" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>9.3096243166515356E-3</v>
       </c>
       <c r="X75" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1.3139243999672293E-2</v>
       </c>
       <c r="Z75" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>2.5912808712802337E-2</v>
       </c>
       <c r="AB75" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>3.0042091244256806E-2</v>
       </c>
     </row>
     <row r="76" spans="9:28" x14ac:dyDescent="0.2">
       <c r="R76" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>4.6146046169639847E-2</v>
       </c>
       <c r="T76" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>9.4551957518150213E-3</v>
       </c>
       <c r="V76" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>5.2498090280974997E-2</v>
       </c>
       <c r="X76" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>3.7376461553716128E-2</v>
       </c>
       <c r="Z76" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>9.584183783495669E-3</v>
       </c>
       <c r="AB76" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1.4461277149981633E-2</v>
       </c>
     </row>
     <row r="77" spans="9:28" x14ac:dyDescent="0.2">
       <c r="R77" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>8.211362349535541E-3</v>
       </c>
       <c r="T77" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1.5382266266781405E-2</v>
       </c>
       <c r="V77" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>7.3478585088140981E-3</v>
       </c>
       <c r="X77" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>5.0975759761370913E-3</v>
       </c>
       <c r="Z77" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1.2399063467501366E-2</v>
       </c>
       <c r="AB77" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1.1159397970513392E-2</v>
       </c>
     </row>
     <row r="78" spans="9:28" x14ac:dyDescent="0.2">
       <c r="R78" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0.7039887103433865</v>
       </c>
       <c r="T78" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>5.7087059856928335E-3</v>
       </c>
       <c r="V78" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0.79336978444361606</v>
       </c>
       <c r="X78" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0.73027778834554646</v>
       </c>
       <c r="Z78" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>4.6019354201572906E-3</v>
       </c>
       <c r="AB78" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>6.8110070967978215E-3</v>
       </c>
     </row>
     <row r="79" spans="9:28" x14ac:dyDescent="0.2">
       <c r="R79" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>3.8340615244731864E-3</v>
       </c>
       <c r="T79" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>4.1810802415572425E-2</v>
       </c>
       <c r="V79" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>3.4397137946801247E-3</v>
       </c>
       <c r="X79" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1.8840279469795964E-3</v>
       </c>
       <c r="Z79" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>3.3701217042322401E-2</v>
       </c>
       <c r="AB79" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>2.9273874524555283E-2</v>
       </c>
     </row>
     <row r="80" spans="9:28" x14ac:dyDescent="0.2">
       <c r="R80" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>8.0556589681991031E-2</v>
       </c>
       <c r="T80" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0.18813754107002503</v>
       </c>
       <c r="V80" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>6.7865301533728439E-2</v>
       </c>
       <c r="X80" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>9.244472086900915E-2</v>
       </c>
       <c r="Z80" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0.19094548473742121</v>
       </c>
       <c r="AB80" s="5">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0.2196385063414531</v>
       </c>
     </row>
@@ -5011,7 +6367,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E243C58-43D1-E447-B84F-2BAE206C52D1}">
-  <dimension ref="E1:Z34"/>
+  <dimension ref="E1:AH40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="7" max="8" width="9" customWidth="1"/>
@@ -5024,11 +6380,13 @@
     <col min="20" max="21" width="10.83203125" style="2"/>
     <col min="22" max="22" width="2.83203125" customWidth="1"/>
     <col min="23" max="24" width="10.83203125" style="2"/>
+    <col min="25" max="25" width="5.6640625" customWidth="1"/>
+    <col min="31" max="31" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="5:26" x14ac:dyDescent="0.2">
+    <row r="1" spans="5:32" x14ac:dyDescent="0.2">
       <c r="H1" s="22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I1" s="22"/>
       <c r="J1" s="22"/>
@@ -5036,44 +6394,25 @@
       <c r="L1" s="23"/>
       <c r="M1" s="21"/>
     </row>
-    <row r="2" spans="5:26" x14ac:dyDescent="0.2">
-      <c r="N2" s="10" t="s">
+    <row r="3" spans="5:32" x14ac:dyDescent="0.2">
+      <c r="H3" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="I3" s="24">
+        <v>4</v>
+      </c>
+      <c r="J3" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="10"/>
-    </row>
-    <row r="3" spans="5:26" x14ac:dyDescent="0.2">
-      <c r="H3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="I3" s="2">
-        <v>4</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="N3" s="10" t="s">
-        <v>9</v>
-      </c>
       <c r="O3" s="10"/>
-      <c r="Q3" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="R3" s="10"/>
-      <c r="T3" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="U3" s="10"/>
-      <c r="W3" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="X3" s="10"/>
-      <c r="Z3" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="5:26" x14ac:dyDescent="0.2">
-      <c r="E4" s="1"/>
+      <c r="AF3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="5:32" x14ac:dyDescent="0.2">
       <c r="H4" s="3" t="s">
         <v>1</v>
       </c>
@@ -5083,11 +6422,33 @@
       <c r="J4" s="16" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="5:26" x14ac:dyDescent="0.2">
+      <c r="N4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="O4" s="10"/>
+      <c r="Q4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="R4" s="10"/>
+      <c r="T4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="U4" s="10"/>
+      <c r="W4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="X4" s="10"/>
+      <c r="Z4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AF4" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="5:32" x14ac:dyDescent="0.2">
       <c r="E5" s="1"/>
       <c r="H5" s="3" t="s">
-        <v>2</v>
+        <v>99</v>
       </c>
       <c r="I5" s="15">
         <v>3</v>
@@ -5095,328 +6456,355 @@
       <c r="J5" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="N5" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="O5" s="9"/>
-      <c r="Z5" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="5:26" x14ac:dyDescent="0.2">
+      <c r="AF5" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="5:32" x14ac:dyDescent="0.2">
+      <c r="E6" s="1"/>
       <c r="H6" s="3" t="s">
-        <v>3</v>
+        <v>89</v>
       </c>
       <c r="I6" s="17">
         <v>4</v>
       </c>
       <c r="J6" s="17"/>
-      <c r="N6" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="O6" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q6" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="R6" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="T6" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="U6" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="W6" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="X6" s="10" t="s">
-        <v>61</v>
-      </c>
+      <c r="N6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="O6" s="9"/>
       <c r="Z6" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" spans="5:26" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+      <c r="AF6" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="5:32" x14ac:dyDescent="0.2">
       <c r="H7" s="3" t="s">
-        <v>53</v>
+        <v>88</v>
       </c>
       <c r="I7" s="18">
         <v>2</v>
       </c>
       <c r="J7" s="18"/>
-      <c r="N7" s="7">
+      <c r="N7" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="O7" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q7" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="R7" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="T7" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="U7" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="W7" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="X7" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF7" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="5:32" x14ac:dyDescent="0.2">
+      <c r="N8" s="7">
         <v>2</v>
       </c>
-      <c r="O7" s="7">
-        <f>N7+1</f>
+      <c r="O8" s="7">
+        <f>N8+1</f>
         <v>3</v>
       </c>
-      <c r="Q7" s="7">
-        <v>1</v>
-      </c>
-      <c r="R7" s="7">
-        <f>Q7+1</f>
+      <c r="Q8" s="7">
+        <v>1</v>
+      </c>
+      <c r="R8" s="7">
+        <f>Q8+1</f>
         <v>2</v>
       </c>
-      <c r="T7" s="7">
-        <v>1</v>
-      </c>
-      <c r="U7" s="7">
-        <f>T7+1</f>
+      <c r="T8" s="7">
+        <v>1</v>
+      </c>
+      <c r="U8" s="7">
+        <f>T8+1</f>
         <v>2</v>
       </c>
-      <c r="W7" s="7">
-        <v>1</v>
-      </c>
-      <c r="X7" s="7">
-        <f>W7+1</f>
+      <c r="W8" s="7">
+        <v>1</v>
+      </c>
+      <c r="X8" s="7">
+        <f>W8+1</f>
         <v>2</v>
       </c>
-      <c r="Z7" s="1" t="s">
+      <c r="Z8" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="8" spans="5:26" x14ac:dyDescent="0.2">
-      <c r="N8" s="7">
-        <v>-1</v>
-      </c>
-      <c r="O8" s="7">
-        <f>N8-1</f>
-        <v>-2</v>
-      </c>
-      <c r="Q8" s="7">
-        <v>0</v>
-      </c>
-      <c r="R8" s="7">
-        <f>Q8-1</f>
-        <v>-1</v>
-      </c>
-      <c r="T8" s="7">
-        <v>1</v>
-      </c>
-      <c r="U8" s="7">
-        <f>T8-1</f>
-        <v>0</v>
-      </c>
-      <c r="W8" s="7">
-        <v>2</v>
-      </c>
-      <c r="X8" s="7">
-        <f>W8-1</f>
-        <v>1</v>
-      </c>
-      <c r="Z8" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="5:26" x14ac:dyDescent="0.2">
-      <c r="I9" s="24" t="str">
+      <c r="AF8" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="5:32" x14ac:dyDescent="0.2">
+      <c r="H9" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="I9" s="9" t="str">
         <f>"(N, L, Hin) = ("&amp;I7&amp;","&amp;I6&amp;","&amp;I3&amp;")"</f>
         <v>(N, L, Hin) = (2,4,4)</v>
       </c>
+      <c r="J9" s="10"/>
       <c r="N9" s="7">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="O9" s="7">
-        <f>N9+1</f>
-        <v>1</v>
+        <f>N9-1</f>
+        <v>-2</v>
       </c>
       <c r="Q9" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R9" s="7">
-        <f>Q9+1</f>
+        <f>Q9-1</f>
+        <v>-1</v>
+      </c>
+      <c r="T9" s="7">
+        <v>1</v>
+      </c>
+      <c r="U9" s="7">
+        <f>T9-1</f>
+        <v>0</v>
+      </c>
+      <c r="W9" s="7">
         <v>2</v>
       </c>
-      <c r="T9" s="7">
-        <v>0</v>
-      </c>
-      <c r="U9" s="7">
-        <f>T9+1</f>
-        <v>1</v>
-      </c>
-      <c r="W9" s="7">
+      <c r="X9" s="7">
+        <f>W9-1</f>
+        <v>1</v>
+      </c>
+      <c r="Z9" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AF9" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="5:32" x14ac:dyDescent="0.2">
+      <c r="H10" s="26" t="s">
+        <v>84</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="J10" s="10"/>
+      <c r="N10" s="7">
+        <v>0</v>
+      </c>
+      <c r="O10" s="7">
+        <f>N10+1</f>
+        <v>1</v>
+      </c>
+      <c r="Q10" s="7">
+        <v>1</v>
+      </c>
+      <c r="R10" s="7">
+        <f>Q10+1</f>
+        <v>2</v>
+      </c>
+      <c r="T10" s="7">
+        <v>0</v>
+      </c>
+      <c r="U10" s="7">
+        <f>T10+1</f>
+        <v>1</v>
+      </c>
+      <c r="W10" s="7">
         <v>-1</v>
       </c>
-      <c r="X9" s="7">
-        <f>W9+1</f>
-        <v>0</v>
-      </c>
-      <c r="Z9" s="1" t="s">
+      <c r="X10" s="7">
+        <f>W10+1</f>
+        <v>0</v>
+      </c>
+      <c r="Z10" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="5:26" x14ac:dyDescent="0.2">
-      <c r="N10" s="7">
-        <v>1</v>
-      </c>
-      <c r="O10" s="7">
-        <f>N10-1</f>
-        <v>0</v>
-      </c>
-      <c r="Q10" s="7">
-        <v>0</v>
-      </c>
-      <c r="R10" s="7">
-        <f>Q10-1</f>
+    <row r="11" spans="5:32" x14ac:dyDescent="0.2">
+      <c r="H11" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="J11" s="10"/>
+      <c r="N11" s="7">
+        <v>1</v>
+      </c>
+      <c r="O11" s="7">
+        <f>N11-1</f>
+        <v>0</v>
+      </c>
+      <c r="Q11" s="7">
+        <v>0</v>
+      </c>
+      <c r="R11" s="7">
+        <f>Q11-1</f>
         <v>-1</v>
       </c>
-      <c r="T10" s="7">
-        <v>0</v>
-      </c>
-      <c r="U10" s="7">
-        <f>T10-1</f>
+      <c r="T11" s="7">
+        <v>0</v>
+      </c>
+      <c r="U11" s="7">
+        <f>T11-1</f>
         <v>-1</v>
       </c>
-      <c r="W10" s="7">
+      <c r="W11" s="7">
         <v>2</v>
       </c>
-      <c r="X10" s="7">
-        <f>W10-1</f>
-        <v>1</v>
-      </c>
-      <c r="Z10" s="1" t="s">
+      <c r="X11" s="7">
+        <f>W11-1</f>
+        <v>1</v>
+      </c>
+      <c r="Z11" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="12" spans="5:26" x14ac:dyDescent="0.2">
-      <c r="N12" s="9" t="s">
+      <c r="AF11" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="5:32" x14ac:dyDescent="0.2">
+      <c r="H12" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="AF12" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="5:32" x14ac:dyDescent="0.2">
+      <c r="N13" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="O12" s="9"/>
-    </row>
-    <row r="13" spans="5:26" x14ac:dyDescent="0.2">
-      <c r="I13" s="9" t="s">
+      <c r="O13" s="9"/>
+      <c r="AA13" t="s">
+        <v>63</v>
+      </c>
+      <c r="AF13" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="5:32" x14ac:dyDescent="0.2">
+      <c r="I14" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="N13" s="10" t="s">
+      <c r="N14" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="O13" s="10" t="s">
+      <c r="O14" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="Q13" s="10" t="s">
+      <c r="Q14" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="R13" s="10" t="s">
+      <c r="R14" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="T13" s="10" t="s">
+      <c r="T14" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="U13" s="10" t="s">
+      <c r="U14" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="W13" s="10" t="s">
+      <c r="W14" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="X13" s="10" t="s">
+      <c r="X14" s="10" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="14" spans="5:26" x14ac:dyDescent="0.2">
-      <c r="I14" s="7">
+      <c r="AF14" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="5:32" x14ac:dyDescent="0.2">
+      <c r="I15" s="7">
         <v>0.37663882999999998</v>
       </c>
-      <c r="J14" s="7">
+      <c r="J15" s="7">
         <v>-0.48650870000000002</v>
       </c>
-      <c r="K14" s="7">
+      <c r="K15" s="7">
         <v>0.40739626000000001</v>
       </c>
-      <c r="L14" s="7">
+      <c r="L15" s="7">
         <v>-0.56883289999999997</v>
       </c>
-      <c r="N14" s="8">
-        <v>0</v>
-      </c>
-      <c r="O14" s="8">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="12">
-        <f>N24</f>
+      <c r="N15" s="8">
+        <v>0</v>
+      </c>
+      <c r="O15" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="12">
+        <f t="shared" ref="Q15:R17" si="0">N25</f>
         <v>0.59702168656330246</v>
       </c>
-      <c r="R14" s="12">
-        <f>O24</f>
+      <c r="R15" s="12">
+        <f t="shared" si="0"/>
         <v>0.98733574020680392</v>
-      </c>
-      <c r="T14" s="12">
-        <f t="shared" ref="T14" si="0">Q24</f>
-        <v>0.74747492715389685</v>
-      </c>
-      <c r="U14" s="12">
-        <f>R24</f>
-        <v>0.98889286311226698</v>
-      </c>
-      <c r="W14" s="12">
-        <f>T24</f>
-        <v>0.2069797447924186</v>
-      </c>
-      <c r="X14" s="12">
-        <f>U24</f>
-        <v>0.93767409884575126</v>
-      </c>
-    </row>
-    <row r="15" spans="5:26" x14ac:dyDescent="0.2">
-      <c r="I15" s="7">
-        <v>0.56738049999999995</v>
-      </c>
-      <c r="J15" s="7">
-        <v>-0.16735654</v>
-      </c>
-      <c r="K15" s="7">
-        <v>-0.15659580000000001</v>
-      </c>
-      <c r="L15" s="7">
-        <v>-0.46818936</v>
-      </c>
-      <c r="N15" s="8">
-        <v>0</v>
-      </c>
-      <c r="O15" s="8">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="12">
-        <f>N25</f>
-        <v>2.1762243525109404E-2</v>
-      </c>
-      <c r="R15" s="12">
-        <f>O25</f>
-        <v>0.78874291389282269</v>
       </c>
       <c r="T15" s="12">
         <f t="shared" ref="T15" si="1">Q25</f>
-        <v>-0.36858254987587874</v>
+        <v>0.74747492715389685</v>
       </c>
       <c r="U15" s="12">
         <f>R25</f>
-        <v>0.66444545594329663</v>
+        <v>0.98889286311226698</v>
       </c>
       <c r="W15" s="12">
-        <f>T25</f>
-        <v>-0.67174814695189922</v>
+        <f t="shared" ref="W15:X17" si="2">T25</f>
+        <v>0.2069797447924186</v>
       </c>
       <c r="X15" s="12">
-        <f>U25</f>
-        <v>0.53843094883651643</v>
-      </c>
-    </row>
-    <row r="16" spans="5:26" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v>0.93767409884575126</v>
+      </c>
+      <c r="Z15" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA15" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB15" s="7">
+        <v>-1</v>
+      </c>
+      <c r="AC15" s="7">
+        <v>0</v>
+      </c>
+      <c r="AD15" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="5:32" x14ac:dyDescent="0.2">
       <c r="I16" s="7">
-        <v>0.13276318000000001</v>
+        <v>0.56738049999999995</v>
       </c>
       <c r="J16" s="7">
-        <v>0.24627653999999999</v>
+        <v>-0.16735654</v>
       </c>
       <c r="K16" s="7">
-        <v>-0.103348464</v>
+        <v>-0.15659580000000001</v>
       </c>
       <c r="L16" s="7">
-        <v>-0.49837208</v>
+        <v>-0.46818936</v>
       </c>
       <c r="N16" s="8">
         <v>0</v>
@@ -5425,386 +6813,629 @@
         <v>0</v>
       </c>
       <c r="Q16" s="12">
-        <f>N26</f>
-        <v>-0.78826169024843407</v>
+        <f t="shared" si="0"/>
+        <v>2.1762243525109404E-2</v>
       </c>
       <c r="R16" s="12">
-        <f>O26</f>
-        <v>-0.65574613778691715</v>
+        <f t="shared" si="0"/>
+        <v>0.78874291389282269</v>
       </c>
       <c r="T16" s="12">
-        <f t="shared" ref="T16" si="2">Q26</f>
-        <v>-0.46423281988402665</v>
+        <f t="shared" ref="T16" si="3">Q26</f>
+        <v>-0.36858254987587874</v>
       </c>
       <c r="U16" s="12">
         <f>R26</f>
+        <v>0.66444545594329663</v>
+      </c>
+      <c r="W16" s="12">
+        <f t="shared" si="2"/>
+        <v>-0.67174814695189922</v>
+      </c>
+      <c r="X16" s="12">
+        <f t="shared" si="2"/>
+        <v>0.53843094883651643</v>
+      </c>
+      <c r="Z16" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA16" s="7">
+        <v>1</v>
+      </c>
+      <c r="AB16" s="7">
+        <v>0</v>
+      </c>
+      <c r="AC16" s="7">
+        <v>1</v>
+      </c>
+      <c r="AD16" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I17" s="7">
+        <v>0.13276318000000001</v>
+      </c>
+      <c r="J17" s="7">
+        <v>0.24627653999999999</v>
+      </c>
+      <c r="K17" s="7">
+        <v>-0.103348464</v>
+      </c>
+      <c r="L17" s="7">
+        <v>-0.49837208</v>
+      </c>
+      <c r="N17" s="8">
+        <v>0</v>
+      </c>
+      <c r="O17" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="12">
+        <f t="shared" si="0"/>
+        <v>-0.78826169024843407</v>
+      </c>
+      <c r="R17" s="12">
+        <f t="shared" si="0"/>
+        <v>-0.65574613778691715</v>
+      </c>
+      <c r="T17" s="12">
+        <f t="shared" ref="T17" si="4">Q27</f>
+        <v>-0.46423281988402665</v>
+      </c>
+      <c r="U17" s="12">
+        <f>R27</f>
         <v>-0.35554650969730994</v>
       </c>
-      <c r="W16" s="12">
-        <f>T26</f>
+      <c r="W17" s="12">
+        <f t="shared" si="2"/>
         <v>-0.30476813848255885</v>
       </c>
-      <c r="X16" s="12">
-        <f>U26</f>
+      <c r="X17" s="12">
+        <f t="shared" si="2"/>
         <v>-0.12043710884126756</v>
       </c>
-    </row>
-    <row r="18" spans="9:24" x14ac:dyDescent="0.2">
-      <c r="I18" s="9" t="s">
+      <c r="Z17" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA17" s="7">
+        <v>1</v>
+      </c>
+      <c r="AB17" s="7">
+        <v>1</v>
+      </c>
+      <c r="AC17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AD17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF17" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="18" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="Z18" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA18" s="7">
+        <v>1</v>
+      </c>
+      <c r="AB18" s="7">
+        <v>2</v>
+      </c>
+      <c r="AC18" s="7">
+        <v>-1</v>
+      </c>
+      <c r="AD18" s="7">
+        <v>2</v>
+      </c>
+      <c r="AF18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="19" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I19" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="N18" s="9" t="s">
+      <c r="N19" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="O18" s="9"/>
-    </row>
-    <row r="19" spans="9:24" x14ac:dyDescent="0.2">
-      <c r="I19" s="8">
+      <c r="O19" s="9"/>
+      <c r="AF19" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I20" s="8">
         <v>0.17738365</v>
       </c>
-      <c r="J19" s="8">
+      <c r="J20" s="8">
         <v>-0.3528347</v>
       </c>
-      <c r="K19" s="8">
+      <c r="K20" s="8">
         <v>-8.5500489999999998E-2</v>
       </c>
-      <c r="N19" s="14" cm="1">
-        <f t="array" ref="N19:O21">MMULT($I$14:$L$16,N7:O10)+MMULT($I$19:$K$21,N14:O16)+MMULT($I$24:$I$26,1)+MMULT($K$24:$K$26,1)</f>
+      <c r="N20" s="14" cm="1">
+        <f t="array" ref="N20:O22">MMULT($I$15:$L$17,N8:O11)+MMULT($I$20:$K$22,N15:O17)+MMULT($I$25:$I$27,1)+MMULT($K$25:$K$27,1)</f>
         <v>0.68850649000000008</v>
       </c>
-      <c r="O19" s="14">
+      <c r="O20" s="14">
         <v>2.5278831800000003</v>
       </c>
-      <c r="Q19" s="14" cm="1">
-        <f t="array" ref="Q19:R21">MMULT($I$14:$L$16,Q7:R10)+MMULT($I$19:$K$21,Q14:R16)+MMULT($I$24:$I$26,1)+MMULT($K$24:$K$26,1)</f>
+      <c r="Q20" s="14" cm="1">
+        <f t="array" ref="Q20:R22">MMULT($I$15:$L$17,Q8:R11)+MMULT($I$20:$K$22,Q15:R17)+MMULT($I$25:$I$27,1)+MMULT($K$25:$K$27,1)</f>
         <v>0.96720829199071501</v>
       </c>
-      <c r="R19" s="14">
+      <c r="R20" s="14">
         <v>2.593872774069224</v>
       </c>
-      <c r="T19" s="14" cm="1">
-        <f t="array" ref="T19:U21">MMULT($I$14:$L$16,T7:U10)+MMULT($I$19:$K$21,T14:U16)+MMULT($I$24:$I$26,1)+MMULT($K$24:$K$26,1)</f>
+      <c r="T20" s="14" cm="1">
+        <f t="array" ref="T20:U22">MMULT($I$15:$L$17,T8:U11)+MMULT($I$20:$K$22,T15:U17)+MMULT($I$25:$I$27,1)+MMULT($K$25:$K$27,1)</f>
         <v>0.21001383784689898</v>
       </c>
-      <c r="U19" s="14">
+      <c r="U20" s="14">
         <v>1.7184332632005979</v>
       </c>
-      <c r="W19" s="14" cm="1">
-        <f t="array" ref="W19:X21">MMULT($I$14:$L$16,W7:X10)+MMULT($I$19:$K$21,W14:X16)+MMULT($I$24:$I$26,1)+MMULT($K$24:$K$26,1)</f>
+      <c r="W20" s="14" cm="1">
+        <f t="array" ref="W20:X22">MMULT($I$15:$L$17,W8:X11)+MMULT($I$20:$K$22,W15:X17)+MMULT($I$25:$I$27,1)+MMULT($K$25:$K$27,1)</f>
         <v>-1.8240988963106761</v>
       </c>
-      <c r="X19" s="14">
+      <c r="X20" s="14">
         <v>-0.2978625463196159</v>
       </c>
-    </row>
-    <row r="20" spans="9:24" x14ac:dyDescent="0.2">
-      <c r="I20" s="8">
+      <c r="Z20" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA20" s="7">
+        <v>3</v>
+      </c>
+      <c r="AB20" s="7">
+        <v>-2</v>
+      </c>
+      <c r="AC20" s="7">
+        <v>1</v>
+      </c>
+      <c r="AD20" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I21" s="8">
         <v>-0.53121185000000004</v>
       </c>
-      <c r="J20" s="8">
+      <c r="J21" s="8">
         <v>0.52461829999999998</v>
       </c>
-      <c r="K20" s="8">
+      <c r="K21" s="8">
         <v>-0.40636771999999999</v>
       </c>
-      <c r="N20" s="14">
+      <c r="N21" s="14">
         <v>2.1765679999999787E-2</v>
       </c>
-      <c r="O20" s="14">
+      <c r="O21" s="14">
         <v>1.06809628</v>
       </c>
-      <c r="Q20" s="14">
+      <c r="Q21" s="14">
         <v>-0.38678181757748087</v>
       </c>
-      <c r="R20" s="14">
+      <c r="R21" s="14">
         <v>0.80073138440839875</v>
       </c>
-      <c r="T20" s="14">
+      <c r="T21" s="14">
         <v>-0.81392199704214296</v>
       </c>
-      <c r="U20" s="14">
+      <c r="U21" s="14">
         <v>0.60194332277368678</v>
       </c>
-      <c r="W20" s="14">
+      <c r="W21" s="14">
         <v>-1.6977915304619624</v>
       </c>
-      <c r="X20" s="14">
+      <c r="X21" s="14">
         <v>-0.47963851037571659</v>
       </c>
-    </row>
-    <row r="21" spans="9:24" x14ac:dyDescent="0.2">
-      <c r="I21" s="8">
+      <c r="Z21" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="AA21" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB21" s="7">
+        <v>-1</v>
+      </c>
+      <c r="AC21" s="7">
+        <v>2</v>
+      </c>
+      <c r="AD21" s="7">
+        <v>-1</v>
+      </c>
+      <c r="AF21" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I22" s="8">
         <v>-0.32683295000000001</v>
       </c>
-      <c r="J21" s="8">
+      <c r="J22" s="8">
         <v>2.4811735000000001E-2</v>
       </c>
-      <c r="K21" s="8">
+      <c r="K22" s="8">
         <v>-0.31738191999999998</v>
       </c>
-      <c r="N21" s="14">
+      <c r="N22" s="14">
         <v>-1.0668240900000001</v>
       </c>
-      <c r="O21" s="14">
+      <c r="O22" s="14">
         <v>-0.78531383399999988</v>
       </c>
-      <c r="Q21" s="14">
+      <c r="Q22" s="14">
         <v>-0.50269350530061574</v>
       </c>
-      <c r="R21" s="14">
+      <c r="R22" s="14">
         <v>-0.37177866220619049</v>
       </c>
-      <c r="T21" s="14">
+      <c r="T22" s="14">
         <v>-0.31476761434408129</v>
       </c>
-      <c r="U21" s="14">
+      <c r="U22" s="14">
         <v>-0.12102454721307829</v>
       </c>
-      <c r="W21" s="14">
+      <c r="W22" s="14">
         <v>-0.84336840664324453</v>
       </c>
-      <c r="X21" s="14">
+      <c r="X22" s="14">
         <v>-0.82914983500272788</v>
       </c>
-    </row>
-    <row r="23" spans="9:24" x14ac:dyDescent="0.2">
-      <c r="I23" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="K23" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="N23" s="9" t="s">
+      <c r="Z22" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="AA22" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB22" s="7">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="7">
+        <v>1</v>
+      </c>
+      <c r="AD22" s="7">
+        <v>-1</v>
+      </c>
+      <c r="AF22" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="Z23" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA23" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB23" s="7">
+        <v>1</v>
+      </c>
+      <c r="AC23" s="7">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF23" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I24" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="K24" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="N24" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="O23" s="9"/>
-    </row>
-    <row r="24" spans="9:24" x14ac:dyDescent="0.2">
-      <c r="I24" s="4">
+      <c r="O24" s="9"/>
+      <c r="AF24" s="27" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="25" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I25" s="4">
         <v>-0.42542717000000002</v>
       </c>
-      <c r="K24" s="4">
+      <c r="K25" s="4">
         <v>0.44298019999999999</v>
       </c>
-      <c r="N24" s="19">
-        <f t="shared" ref="N24:O26" si="3">TANH(N19)</f>
+      <c r="N25" s="19">
+        <f t="shared" ref="N25:O27" si="5">TANH(N20)</f>
         <v>0.59702168656330246</v>
       </c>
-      <c r="O24" s="19">
-        <f t="shared" si="3"/>
+      <c r="O25" s="19">
+        <f t="shared" si="5"/>
         <v>0.98733574020680392</v>
-      </c>
-      <c r="P24" s="20"/>
-      <c r="Q24" s="19">
-        <f t="shared" ref="Q24:X24" si="4">TANH(Q19)</f>
-        <v>0.74747492715389685</v>
-      </c>
-      <c r="R24" s="19">
-        <f t="shared" si="4"/>
-        <v>0.98889286311226698</v>
-      </c>
-      <c r="S24" s="20"/>
-      <c r="T24" s="19">
-        <f t="shared" si="4"/>
-        <v>0.2069797447924186</v>
-      </c>
-      <c r="U24" s="19">
-        <f t="shared" si="4"/>
-        <v>0.93767409884575126</v>
-      </c>
-      <c r="V24" s="20"/>
-      <c r="W24" s="19">
-        <f t="shared" si="4"/>
-        <v>-0.94924552092215564</v>
-      </c>
-      <c r="X24" s="19">
-        <f t="shared" si="4"/>
-        <v>-0.28935533383199491</v>
-      </c>
-    </row>
-    <row r="25" spans="9:24" x14ac:dyDescent="0.2">
-      <c r="I25" s="4">
-        <v>-0.45248749999999999</v>
-      </c>
-      <c r="K25" s="4">
-        <v>-0.35967500000000002</v>
-      </c>
-      <c r="N25" s="19">
-        <f t="shared" si="3"/>
-        <v>2.1762243525109404E-2</v>
-      </c>
-      <c r="O25" s="19">
-        <f t="shared" ref="O25:X25" si="5">TANH(O20)</f>
-        <v>0.78874291389282269</v>
       </c>
       <c r="P25" s="20"/>
       <c r="Q25" s="19">
-        <f t="shared" si="5"/>
-        <v>-0.36858254987587874</v>
+        <f t="shared" ref="Q25:X25" si="6">TANH(Q20)</f>
+        <v>0.74747492715389685</v>
       </c>
       <c r="R25" s="19">
-        <f t="shared" si="5"/>
-        <v>0.66444545594329663</v>
+        <f t="shared" si="6"/>
+        <v>0.98889286311226698</v>
       </c>
       <c r="S25" s="20"/>
       <c r="T25" s="19">
+        <f t="shared" si="6"/>
+        <v>0.2069797447924186</v>
+      </c>
+      <c r="U25" s="19">
+        <f t="shared" si="6"/>
+        <v>0.93767409884575126</v>
+      </c>
+      <c r="V25" s="20"/>
+      <c r="W25" s="29">
+        <f t="shared" si="6"/>
+        <v>-0.94924552092215564</v>
+      </c>
+      <c r="X25" s="29">
+        <f t="shared" si="6"/>
+        <v>-0.28935533383199491</v>
+      </c>
+    </row>
+    <row r="26" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I26" s="4">
+        <v>-0.45248749999999999</v>
+      </c>
+      <c r="K26" s="4">
+        <v>-0.35967500000000002</v>
+      </c>
+      <c r="N26" s="19">
         <f t="shared" si="5"/>
-        <v>-0.67174814695189922</v>
-      </c>
-      <c r="U25" s="19">
-        <f t="shared" si="5"/>
-        <v>0.53843094883651643</v>
-      </c>
-      <c r="V25" s="20"/>
-      <c r="W25" s="19">
-        <f t="shared" si="5"/>
-        <v>-0.93513241904863653</v>
-      </c>
-      <c r="X25" s="19">
-        <f t="shared" si="5"/>
-        <v>-0.44595405857219844</v>
-      </c>
-    </row>
-    <row r="26" spans="9:24" x14ac:dyDescent="0.2">
-      <c r="I26" s="4">
-        <v>-0.41191080000000002</v>
-      </c>
-      <c r="K26" s="4">
-        <v>-0.17579102999999999</v>
-      </c>
-      <c r="N26" s="19">
-        <f t="shared" si="3"/>
-        <v>-0.78826169024843407</v>
+        <v>2.1762243525109404E-2</v>
       </c>
       <c r="O26" s="19">
-        <f t="shared" ref="O26:X26" si="6">TANH(O21)</f>
-        <v>-0.65574613778691715</v>
+        <f t="shared" ref="O26:X26" si="7">TANH(O21)</f>
+        <v>0.78874291389282269</v>
       </c>
       <c r="P26" s="20"/>
       <c r="Q26" s="19">
-        <f t="shared" si="6"/>
-        <v>-0.46423281988402665</v>
+        <f t="shared" si="7"/>
+        <v>-0.36858254987587874</v>
       </c>
       <c r="R26" s="19">
-        <f t="shared" si="6"/>
-        <v>-0.35554650969730994</v>
+        <f t="shared" si="7"/>
+        <v>0.66444545594329663</v>
       </c>
       <c r="S26" s="20"/>
       <c r="T26" s="19">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
+        <v>-0.67174814695189922</v>
+      </c>
+      <c r="U26" s="19">
+        <f t="shared" si="7"/>
+        <v>0.53843094883651643</v>
+      </c>
+      <c r="V26" s="20"/>
+      <c r="W26" s="29">
+        <f t="shared" si="7"/>
+        <v>-0.93513241904863653</v>
+      </c>
+      <c r="X26" s="29">
+        <f t="shared" si="7"/>
+        <v>-0.44595405857219844</v>
+      </c>
+      <c r="AF26" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="27" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I27" s="4">
+        <v>-0.41191080000000002</v>
+      </c>
+      <c r="K27" s="4">
+        <v>-0.17579102999999999</v>
+      </c>
+      <c r="N27" s="19">
+        <f t="shared" si="5"/>
+        <v>-0.78826169024843407</v>
+      </c>
+      <c r="O27" s="19">
+        <f t="shared" ref="O27:X27" si="8">TANH(O22)</f>
+        <v>-0.65574613778691715</v>
+      </c>
+      <c r="P27" s="20"/>
+      <c r="Q27" s="19">
+        <f t="shared" si="8"/>
+        <v>-0.46423281988402665</v>
+      </c>
+      <c r="R27" s="19">
+        <f t="shared" si="8"/>
+        <v>-0.35554650969730994</v>
+      </c>
+      <c r="S27" s="20"/>
+      <c r="T27" s="19">
+        <f t="shared" si="8"/>
         <v>-0.30476813848255885</v>
       </c>
-      <c r="U26" s="19">
-        <f t="shared" si="6"/>
+      <c r="U27" s="19">
+        <f t="shared" si="8"/>
         <v>-0.12043710884126756</v>
       </c>
-      <c r="V26" s="20"/>
-      <c r="W26" s="19">
-        <f t="shared" si="6"/>
+      <c r="V27" s="20"/>
+      <c r="W27" s="29">
+        <f t="shared" si="8"/>
         <v>-0.68758907375906397</v>
       </c>
-      <c r="X26" s="19">
-        <f t="shared" si="6"/>
+      <c r="X27" s="29">
+        <f t="shared" si="8"/>
         <v>-0.68001924383799983</v>
       </c>
-    </row>
-    <row r="29" spans="9:24" x14ac:dyDescent="0.2">
-      <c r="I29" s="9" t="s">
+      <c r="AA27" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="AF27" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="AG27" s="28"/>
+      <c r="AH27" s="28"/>
+    </row>
+    <row r="28" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="AF28" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="AF29" s="27" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="30" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I30" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="N29" s="9" t="s">
+      <c r="N30" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="O29" s="9"/>
-    </row>
-    <row r="30" spans="9:24" x14ac:dyDescent="0.2">
-      <c r="I30" s="11">
+      <c r="O30" s="9"/>
+      <c r="AF30" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="31" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I31" s="11">
         <v>3</v>
       </c>
-      <c r="J30" s="11">
-        <v>0</v>
-      </c>
-      <c r="K30" s="11">
+      <c r="J31" s="11">
+        <v>0</v>
+      </c>
+      <c r="K31" s="11">
         <v>-1</v>
       </c>
-      <c r="N30" s="5" cm="1">
-        <f t="array" ref="N30:O30">MMULT($I$30:$K$30,N24:O26)+MMULT($I$34,1)</f>
+      <c r="N31" s="5" cm="1">
+        <f t="array" ref="N31:O31">MMULT($I$31:$K$31,N25:O27)+MMULT($I$35,1)</f>
         <v>5.5793267499383417</v>
       </c>
-      <c r="O30" s="5">
+      <c r="O31" s="5">
         <v>6.6177533584073291</v>
       </c>
-      <c r="Q30" s="5" cm="1">
-        <f t="array" ref="Q30:R30">MMULT($I$30:$K$30,Q24:R26)+MMULT($I$34,1)</f>
+      <c r="Q31" s="5" cm="1">
+        <f t="array" ref="Q31:R31">MMULT($I$31:$K$31,Q25:R27)+MMULT($I$35,1)</f>
         <v>5.7066576013457171</v>
       </c>
-      <c r="R30" s="5">
+      <c r="R31" s="5">
         <v>6.3222250990341111</v>
       </c>
-      <c r="T30" s="5" cm="1">
-        <f t="array" ref="T30:U30">MMULT($I$30:$K$30,T24:U26)+MMULT($I$34,1)</f>
+      <c r="T31" s="5" cm="1">
+        <f t="array" ref="T31:U31">MMULT($I$31:$K$31,T25:U27)+MMULT($I$35,1)</f>
         <v>3.9257073728598146</v>
       </c>
-      <c r="U30" s="5">
+      <c r="U31" s="5">
         <v>5.933459405378521</v>
       </c>
-      <c r="W30" s="5" cm="1">
-        <f t="array" ref="W30:X30">MMULT($I$30:$K$30,W24:X26)+MMULT($I$34,1)</f>
+      <c r="W31" s="5" cm="1">
+        <f t="array" ref="W31:X31">MMULT($I$31:$K$31,W25:X27)+MMULT($I$35,1)</f>
         <v>0.83985251099259717</v>
       </c>
-      <c r="X30" s="5">
+      <c r="X31" s="5">
         <v>2.8119532423420153</v>
       </c>
     </row>
-    <row r="33" spans="9:24" x14ac:dyDescent="0.2">
-      <c r="I33" s="9" t="s">
+    <row r="32" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="AG32" s="28"/>
+      <c r="AH32" s="28"/>
+    </row>
+    <row r="33" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="AF33" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="34" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I34" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="N33" s="10" t="s">
+      <c r="N34" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="O33" s="10"/>
-    </row>
-    <row r="34" spans="9:24" x14ac:dyDescent="0.2">
-      <c r="I34" s="4">
+      <c r="O34" s="10"/>
+      <c r="AF34" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="35" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="I35" s="4">
         <v>3</v>
       </c>
-      <c r="N34" s="6">
-        <f>1/(1+EXP(-N30))</f>
+      <c r="N35" s="6">
+        <f>1/(1+EXP(-N31))</f>
         <v>0.99623909157497625</v>
       </c>
-      <c r="O34" s="6">
-        <f>1/(1+EXP(-O30))</f>
+      <c r="O35" s="6">
+        <f>1/(1+EXP(-O31))</f>
         <v>0.99866535360681541</v>
       </c>
-      <c r="Q34" s="6">
-        <f t="shared" ref="Q34:X34" si="7">1/(1+EXP(-Q30))</f>
+      <c r="Q35" s="6">
+        <f t="shared" ref="Q35:X35" si="9">1/(1+EXP(-Q31))</f>
         <v>0.99668724746367743</v>
       </c>
-      <c r="R34" s="6">
-        <f t="shared" si="7"/>
+      <c r="R35" s="6">
+        <f t="shared" si="9"/>
         <v>0.99820727672246345</v>
       </c>
-      <c r="T34" s="6">
-        <f t="shared" si="7"/>
+      <c r="T35" s="6">
+        <f t="shared" si="9"/>
         <v>0.98065349452195583</v>
       </c>
-      <c r="U34" s="6">
-        <f t="shared" si="7"/>
+      <c r="U35" s="6">
+        <f t="shared" si="9"/>
         <v>0.997357699139376</v>
       </c>
-      <c r="W34" s="6">
-        <f t="shared" si="7"/>
+      <c r="W35" s="6">
+        <f t="shared" si="9"/>
         <v>0.69843415220367056</v>
       </c>
-      <c r="X34" s="6">
-        <f t="shared" si="7"/>
+      <c r="X35" s="6">
+        <f t="shared" si="9"/>
         <v>0.9433183472777642</v>
       </c>
+      <c r="AF35" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="AF36" s="27" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="37" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="AF37" s="27" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="38" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="AF38" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="39" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="AG39" s="28"/>
+      <c r="AH39" s="28"/>
+    </row>
+    <row r="40" spans="9:34" x14ac:dyDescent="0.2">
+      <c r="AG40" s="28"/>
+      <c r="AH40" s="28"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="AA27" r:id="rId1" xr:uid="{AD2D0CB1-8A19-3341-960F-D9C9301DE375}"/>
+    <hyperlink ref="H12" r:id="rId2" xr:uid="{41CFA377-33A1-E84F-93B1-A730A074CFCC}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>